<commit_message>
Correct KCNQ1 Lauren analysis with paired patient tests
</commit_message>
<xml_diff>
--- a/outputs/final/kcnq1_lauren_downsampled/KCNQ1_lauren_downsampled_analysis.xlsx
+++ b/outputs/final/kcnq1_lauren_downsampled/KCNQ1_lauren_downsampled_analysis.xlsx
@@ -57,10 +57,10 @@
     <t>Random downsampling to 3368 cells per group, matching the smallest group</t>
   </si>
   <si>
-    <t>Wilcoxon/Mann-Whitney on log1p(CPM), KCNQ1-positive cells only</t>
+    <t>Exploratory Wilcoxon/Mann-Whitney on log1p(CP10K), KCNQ1-positive cells only</t>
   </si>
   <si>
-    <t>Fisher exact test on KCNQ1-positive versus KCNQ1-negative cells</t>
+    <t>Exploratory Fisher exact test on pooled KCNQ1-positive versus KCNQ1-negative cells</t>
   </si>
   <si>
     <t>group</t>
@@ -84,7 +84,7 @@
     <t>mean_raw_per_cell</t>
   </si>
   <si>
-    <t>mean_log1p_cpm_all_cells</t>
+    <t>mean_log1p_cp10k_all_cells</t>
   </si>
   <si>
     <t>n_kcnq1_positive</t>
@@ -96,10 +96,10 @@
     <t>median_raw_among_kcnq1_positive</t>
   </si>
   <si>
-    <t>mean_log1p_cpm_among_kcnq1_positive</t>
+    <t>mean_log1p_cp10k_among_kcnq1_positive</t>
   </si>
   <si>
-    <t>median_log1p_cpm_among_kcnq1_positive</t>
+    <t>median_log1p_cp10k_among_kcnq1_positive</t>
   </si>
   <si>
     <t>Primary normal epithelial</t>
@@ -132,10 +132,10 @@
     <t>group_2_detection_pct</t>
   </si>
   <si>
-    <t>group_1_mean_log1p_cpm_among_positive</t>
+    <t>group_1_mean_log1p_cp10k_among_positive</t>
   </si>
   <si>
-    <t>group_2_mean_log1p_cpm_among_positive</t>
+    <t>group_2_mean_log1p_cp10k_among_positive</t>
   </si>
   <si>
     <t>fisher_fdr_detection</t>
@@ -175,8 +175,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -192,7 +200,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -200,12 +208,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -504,10 +530,10 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
@@ -578,43 +604,43 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:13">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -752,43 +778,43 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:13">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -926,37 +952,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1076,22 +1102,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1406,31 +1432,31 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>26</v>
       </c>
     </row>

</xml_diff>